<commit_message>
Updating the application title
</commit_message>
<xml_diff>
--- a/WBS.xlsx
+++ b/WBS.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="12276" windowHeight="9000"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,9 +27,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="62">
-  <si>
-    <t>Save Plate</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="62">
+  <si>
+    <t>EcoPantry</t>
   </si>
   <si>
     <t>Task No</t>
@@ -225,7 +225,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -266,13 +266,6 @@
       <color theme="1"/>
       <name val="Microsoft YaHei"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -910,152 +903,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="15" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1070,9 +1063,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1100,9 +1090,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1121,19 +1108,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1590,7 +1568,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O52"/>
+  <dimension ref="C5:O52"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="8.53703703703704" customWidth="1"/>
@@ -1605,12 +1583,7 @@
     <col min="11" max="11" width="18.3425925925926" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" ht="28.5" customHeight="1" spans="1:15">
+    <row r="5" ht="28.5" customHeight="1" spans="3:15">
       <c r="C5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1624,862 +1597,862 @@
       <c r="K5" s="1"/>
       <c r="O5" s="2"/>
     </row>
-    <row r="6" ht="22.5" customHeight="1" spans="1:15">
+    <row r="6" ht="22.5" customHeight="1" spans="3:15">
       <c r="C6" s="3"/>
       <c r="D6" s="4"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
     </row>
-    <row r="7" ht="39" customHeight="1" spans="1:15">
-      <c r="C7" s="7" t="s">
+    <row r="7" ht="39" customHeight="1" spans="3:15">
+      <c r="C7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="8"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="10" t="s">
+      <c r="E7" s="7"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="I7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="K7" s="11" t="s">
+      <c r="K7" s="10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1" spans="1:15">
-      <c r="C8" s="12">
+    <row r="8" ht="22.5" customHeight="1" spans="3:15">
+      <c r="C8" s="11">
         <v>1</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="13"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
-    </row>
-    <row r="9" ht="22.5" customHeight="1" spans="1:15">
-      <c r="C9" s="17"/>
-      <c r="D9" s="18">
+      <c r="E8" s="12"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+    </row>
+    <row r="9" ht="22.5" customHeight="1" spans="3:15">
+      <c r="C9" s="15"/>
+      <c r="D9" s="16">
         <v>1.1</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="15">
+      <c r="F9" s="17"/>
+      <c r="G9" s="14">
         <v>1</v>
       </c>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16">
-        <v>100</v>
-      </c>
-      <c r="J9" s="16">
-        <v>100</v>
-      </c>
-      <c r="K9" s="16">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" ht="22.5" customHeight="1" spans="1:15">
-      <c r="C10" s="20"/>
-      <c r="D10" s="21">
+      <c r="H9" s="4"/>
+      <c r="I9" s="4">
+        <v>100</v>
+      </c>
+      <c r="J9" s="4">
+        <v>100</v>
+      </c>
+      <c r="K9" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1" spans="3:15">
+      <c r="C10" s="18"/>
+      <c r="D10" s="19">
         <v>1.2</v>
       </c>
-      <c r="E10" s="21" t="s">
+      <c r="E10" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="16"/>
-    </row>
-    <row r="11" ht="22.5" customHeight="1" spans="1:15">
-      <c r="C11" s="17"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="23" t="s">
+      <c r="F10" s="20"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+    </row>
+    <row r="11" ht="22.5" customHeight="1" spans="3:15">
+      <c r="C11" s="15"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="14">
         <v>1</v>
       </c>
-      <c r="H11" s="16">
+      <c r="H11" s="4">
         <v>1.1</v>
       </c>
-      <c r="I11" s="16">
-        <v>100</v>
-      </c>
-      <c r="J11" s="16">
-        <v>100</v>
-      </c>
-      <c r="K11" s="16">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" ht="22.5" customHeight="1" spans="1:15">
-      <c r="C12" s="20"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="24" t="s">
+      <c r="I11" s="4">
+        <v>100</v>
+      </c>
+      <c r="J11" s="4">
+        <v>100</v>
+      </c>
+      <c r="K11" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" ht="22.5" customHeight="1" spans="3:15">
+      <c r="C12" s="18"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="F12" s="22" t="s">
+      <c r="F12" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="15">
+      <c r="G12" s="14">
         <v>1</v>
       </c>
-      <c r="H12" s="16">
+      <c r="H12" s="4">
         <v>1.1</v>
       </c>
-      <c r="I12" s="16">
-        <v>100</v>
-      </c>
-      <c r="J12" s="16">
-        <v>100</v>
-      </c>
-      <c r="K12" s="16">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="13" ht="22.5" customHeight="1" spans="1:15">
-      <c r="C13" s="17"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="23" t="s">
+      <c r="I12" s="4">
+        <v>100</v>
+      </c>
+      <c r="J12" s="4">
+        <v>100</v>
+      </c>
+      <c r="K12" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" ht="22.5" customHeight="1" spans="3:15">
+      <c r="C13" s="15"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="15">
+      <c r="G13" s="14">
         <v>1</v>
       </c>
-      <c r="H13" s="16">
+      <c r="H13" s="4">
         <v>1.1</v>
       </c>
-      <c r="I13" s="16">
-        <v>100</v>
-      </c>
-      <c r="J13" s="16">
-        <v>100</v>
-      </c>
-      <c r="K13" s="16">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" ht="22.5" customHeight="1" spans="1:15">
-      <c r="C14" s="20"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="26"/>
-    </row>
-    <row r="15" ht="22.5" customHeight="1" spans="1:15">
-      <c r="C15" s="17">
+      <c r="I13" s="4">
+        <v>100</v>
+      </c>
+      <c r="J13" s="4">
+        <v>100</v>
+      </c>
+      <c r="K13" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" ht="22.5" customHeight="1" spans="3:15">
+      <c r="C14" s="18"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="22"/>
+      <c r="J14" s="22"/>
+      <c r="K14" s="22"/>
+    </row>
+    <row r="15" ht="22.5" customHeight="1" spans="3:15">
+      <c r="C15" s="15">
         <v>2</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="18"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
-    </row>
-    <row r="16" ht="22.5" customHeight="1" spans="1:15">
-      <c r="C16" s="20"/>
-      <c r="D16" s="21">
+      <c r="E15" s="16"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+    </row>
+    <row r="16" ht="22.5" customHeight="1" spans="3:15">
+      <c r="C16" s="18"/>
+      <c r="D16" s="19">
         <v>2.1</v>
       </c>
-      <c r="E16" s="24" t="s">
+      <c r="E16" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="22"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
     </row>
     <row r="17" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C17" s="17"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="23" t="s">
+      <c r="C17" s="15"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="F17" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="G17" s="15">
+      <c r="G17" s="14">
         <v>3</v>
       </c>
-      <c r="H17" s="27" t="s">
+      <c r="H17" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I17" s="16">
-        <v>100</v>
-      </c>
-      <c r="J17" s="16"/>
-      <c r="K17" s="16"/>
+      <c r="I17" s="4">
+        <v>100</v>
+      </c>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
     </row>
     <row r="18" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C18" s="20"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="24" t="s">
+      <c r="C18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="22" t="s">
+      <c r="F18" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="G18" s="15">
+      <c r="G18" s="14">
         <v>2</v>
       </c>
-      <c r="H18" s="27" t="s">
+      <c r="H18" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16">
-        <v>100</v>
-      </c>
-      <c r="K18" s="16"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4">
+        <v>100</v>
+      </c>
+      <c r="K18" s="4"/>
     </row>
     <row r="19" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C19" s="17"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="23" t="s">
+      <c r="C19" s="15"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="F19" s="19" t="s">
+      <c r="F19" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="G19" s="15">
+      <c r="G19" s="14">
         <v>2</v>
       </c>
-      <c r="H19" s="27" t="s">
+      <c r="H19" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="16"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="16">
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4">
         <v>100</v>
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C20" s="20"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="26"/>
-      <c r="K20" s="26"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
     </row>
     <row r="21" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C21" s="17"/>
-      <c r="D21" s="18">
+      <c r="C21" s="15"/>
+      <c r="D21" s="16">
         <v>2.2</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="E21" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="F21" s="19"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="16"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="16"/>
-      <c r="K21" s="16"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
     </row>
     <row r="22" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C22" s="20"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="24" t="s">
+      <c r="C22" s="18"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="F22" s="22" t="s">
+      <c r="F22" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="G22" s="15">
+      <c r="G22" s="14">
         <v>3</v>
       </c>
-      <c r="H22" s="27" t="s">
+      <c r="H22" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="I22" s="16">
+      <c r="I22" s="4">
         <v>50</v>
       </c>
-      <c r="J22" s="16"/>
-      <c r="K22" s="16">
+      <c r="J22" s="4"/>
+      <c r="K22" s="4">
         <v>50</v>
       </c>
     </row>
     <row r="23" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C23" s="17"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="23" t="s">
+      <c r="C23" s="15"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="F23" s="19" t="s">
+      <c r="F23" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="15">
+      <c r="G23" s="14">
         <v>4</v>
       </c>
-      <c r="H23" s="27" t="s">
+      <c r="H23" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="I23" s="16"/>
-      <c r="J23" s="16">
-        <v>100</v>
-      </c>
-      <c r="K23" s="16"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4">
+        <v>100</v>
+      </c>
+      <c r="K23" s="4"/>
     </row>
     <row r="24" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C24" s="20"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="26"/>
-      <c r="I24" s="26"/>
-      <c r="J24" s="26"/>
-      <c r="K24" s="26"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="22"/>
+      <c r="J24" s="22"/>
+      <c r="K24" s="22"/>
     </row>
     <row r="25" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C25" s="17">
+      <c r="C25" s="15">
         <v>3</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="D25" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="E25" s="18"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
     </row>
     <row r="26" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C26" s="20"/>
-      <c r="D26" s="21">
+      <c r="C26" s="18"/>
+      <c r="D26" s="19">
         <v>3.1</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="E26" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="F26" s="22"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="16"/>
-      <c r="J26" s="16"/>
-      <c r="K26" s="16"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
     </row>
     <row r="27" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C27" s="17"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="23" t="s">
+      <c r="C27" s="15"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="F27" s="19" t="s">
+      <c r="F27" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="G27" s="15">
+      <c r="G27" s="14">
         <v>3</v>
       </c>
-      <c r="H27" s="27" t="s">
+      <c r="H27" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="I27" s="16">
-        <v>100</v>
-      </c>
-      <c r="J27" s="16"/>
-      <c r="K27" s="16"/>
+      <c r="I27" s="4">
+        <v>100</v>
+      </c>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
     </row>
     <row r="28" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C28" s="20"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="24" t="s">
+      <c r="C28" s="18"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="F28" s="22" t="s">
+      <c r="F28" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="G28" s="15">
+      <c r="G28" s="14">
         <v>2</v>
       </c>
-      <c r="H28" s="27" t="s">
+      <c r="H28" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="I28" s="16">
-        <v>100</v>
-      </c>
-      <c r="J28" s="16"/>
-      <c r="K28" s="16"/>
+      <c r="I28" s="4">
+        <v>100</v>
+      </c>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
     </row>
     <row r="29" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C29" s="17"/>
-      <c r="D29" s="18">
+      <c r="C29" s="15"/>
+      <c r="D29" s="16">
         <v>3.2</v>
       </c>
-      <c r="E29" s="23" t="s">
+      <c r="E29" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="F29" s="19"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
-      <c r="K29" s="16"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
     </row>
     <row r="30" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C30" s="20"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="24" t="s">
+      <c r="C30" s="18"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="F30" s="22" t="s">
+      <c r="F30" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="G30" s="15">
+      <c r="G30" s="14">
         <v>3</v>
       </c>
-      <c r="H30" s="27" t="s">
+      <c r="H30" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16">
-        <v>100</v>
-      </c>
-      <c r="K30" s="16"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4">
+        <v>100</v>
+      </c>
+      <c r="K30" s="4"/>
     </row>
     <row r="31" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C31" s="17"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="23" t="s">
+      <c r="C31" s="15"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="F31" s="19" t="s">
+      <c r="F31" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="G31" s="15">
+      <c r="G31" s="14">
         <v>3</v>
       </c>
-      <c r="H31" s="27" t="s">
+      <c r="H31" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="I31" s="16"/>
-      <c r="J31" s="16">
-        <v>100</v>
-      </c>
-      <c r="K31" s="16"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4">
+        <v>100</v>
+      </c>
+      <c r="K31" s="4"/>
     </row>
     <row r="32" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C32" s="20"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="24" t="s">
+      <c r="C32" s="18"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="F32" s="22" t="s">
+      <c r="F32" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="G32" s="15">
+      <c r="G32" s="14">
         <v>2</v>
       </c>
-      <c r="H32" s="27" t="s">
+      <c r="H32" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="I32" s="16"/>
-      <c r="J32" s="16"/>
-      <c r="K32" s="16">
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4">
         <v>100</v>
       </c>
     </row>
     <row r="33" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C33" s="17"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="26"/>
-      <c r="K33" s="26"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="22"/>
+      <c r="I33" s="22"/>
+      <c r="J33" s="22"/>
+      <c r="K33" s="22"/>
     </row>
     <row r="34" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C34" s="20"/>
-      <c r="D34" s="21">
+      <c r="C34" s="18"/>
+      <c r="D34" s="19">
         <v>3.3</v>
       </c>
-      <c r="E34" s="24" t="s">
+      <c r="E34" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="F34" s="22"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="16"/>
-      <c r="J34" s="16"/>
-      <c r="K34" s="16"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
     </row>
     <row r="35" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C35" s="17"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="23" t="s">
+      <c r="C35" s="15"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="F35" s="19" t="s">
+      <c r="F35" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="G35" s="15">
+      <c r="G35" s="14">
         <v>3</v>
       </c>
-      <c r="H35" s="27" t="s">
+      <c r="H35" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16">
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4">
         <v>100</v>
       </c>
     </row>
     <row r="36" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C36" s="20"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="24" t="s">
+      <c r="C36" s="18"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="F36" s="22" t="s">
+      <c r="F36" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="G36" s="15">
+      <c r="G36" s="14">
         <v>3</v>
       </c>
-      <c r="H36" s="27" t="s">
+      <c r="H36" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="I36" s="16">
-        <v>100</v>
-      </c>
-      <c r="J36" s="16"/>
-      <c r="K36" s="16"/>
+      <c r="I36" s="4">
+        <v>100</v>
+      </c>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
     </row>
     <row r="37" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C37" s="17"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="25"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="26"/>
-      <c r="K37" s="26"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="21"/>
+      <c r="H37" s="22"/>
+      <c r="I37" s="22"/>
+      <c r="J37" s="22"/>
+      <c r="K37" s="22"/>
     </row>
     <row r="38" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C38" s="20"/>
-      <c r="D38" s="21">
+      <c r="C38" s="18"/>
+      <c r="D38" s="19">
         <v>3.4</v>
       </c>
-      <c r="E38" s="24" t="s">
+      <c r="E38" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="F38" s="22"/>
-      <c r="G38" s="15"/>
-      <c r="H38" s="16"/>
-      <c r="I38" s="16"/>
-      <c r="J38" s="16"/>
-      <c r="K38" s="16"/>
+      <c r="F38" s="20"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="4"/>
+      <c r="I38" s="4"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="4"/>
     </row>
     <row r="39" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C39" s="17"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="23" t="s">
+      <c r="C39" s="15"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="F39" s="19" t="s">
+      <c r="F39" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="G39" s="15">
+      <c r="G39" s="14">
         <v>3</v>
       </c>
-      <c r="H39" s="27" t="s">
+      <c r="H39" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="I39" s="16"/>
-      <c r="J39" s="16">
-        <v>100</v>
-      </c>
-      <c r="K39" s="16"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4">
+        <v>100</v>
+      </c>
+      <c r="K39" s="4"/>
     </row>
     <row r="40" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C40" s="20"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="24" t="s">
+      <c r="C40" s="18"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="F40" s="22" t="s">
+      <c r="F40" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="G40" s="15">
+      <c r="G40" s="14">
         <v>3</v>
       </c>
-      <c r="H40" s="27" t="s">
+      <c r="H40" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="I40" s="16"/>
-      <c r="J40" s="16"/>
-      <c r="K40" s="16">
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="4">
         <v>100</v>
       </c>
     </row>
     <row r="41" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C41" s="17"/>
-      <c r="D41" s="18"/>
-      <c r="E41" s="18"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="25"/>
-      <c r="H41" s="26"/>
-      <c r="I41" s="26"/>
-      <c r="J41" s="26"/>
-      <c r="K41" s="26"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="16"/>
+      <c r="E41" s="16"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="21"/>
+      <c r="H41" s="22"/>
+      <c r="I41" s="22"/>
+      <c r="J41" s="22"/>
+      <c r="K41" s="22"/>
     </row>
     <row r="42" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C42" s="20"/>
-      <c r="D42" s="21"/>
-      <c r="E42" s="21"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="25"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="26"/>
-      <c r="J42" s="26"/>
-      <c r="K42" s="26"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="19"/>
+      <c r="E42" s="19"/>
+      <c r="F42" s="20"/>
+      <c r="G42" s="21"/>
+      <c r="H42" s="22"/>
+      <c r="I42" s="22"/>
+      <c r="J42" s="22"/>
+      <c r="K42" s="22"/>
     </row>
     <row r="43" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C43" s="17">
+      <c r="C43" s="15">
         <v>4</v>
       </c>
-      <c r="D43" s="18" t="s">
+      <c r="D43" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="E43" s="18"/>
-      <c r="F43" s="19"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="16"/>
-      <c r="I43" s="16"/>
-      <c r="J43" s="16"/>
-      <c r="K43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="F43" s="17"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="4"/>
     </row>
     <row r="44" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C44" s="20"/>
-      <c r="D44" s="21">
+      <c r="C44" s="18"/>
+      <c r="D44" s="19">
         <v>4.1</v>
       </c>
-      <c r="E44" s="21" t="s">
+      <c r="E44" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F44" s="22"/>
-      <c r="G44" s="15">
+      <c r="F44" s="20"/>
+      <c r="G44" s="14">
         <v>2</v>
       </c>
-      <c r="H44" s="27" t="s">
+      <c r="H44" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="I44" s="16">
+      <c r="I44" s="4">
         <v>50</v>
       </c>
-      <c r="J44" s="16">
+      <c r="J44" s="4">
         <v>50</v>
       </c>
-      <c r="K44" s="16"/>
+      <c r="K44" s="4"/>
     </row>
     <row r="45" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C45" s="17"/>
-      <c r="D45" s="18">
+      <c r="C45" s="15"/>
+      <c r="D45" s="16">
         <v>4.2</v>
       </c>
-      <c r="E45" s="18" t="s">
+      <c r="E45" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="F45" s="19"/>
-      <c r="G45" s="15">
+      <c r="F45" s="17"/>
+      <c r="G45" s="14">
         <v>2</v>
       </c>
-      <c r="H45" s="16">
+      <c r="H45" s="4">
         <v>4.1</v>
       </c>
-      <c r="I45" s="16">
+      <c r="I45" s="4">
         <v>50</v>
       </c>
-      <c r="J45" s="16"/>
-      <c r="K45" s="16">
+      <c r="J45" s="4"/>
+      <c r="K45" s="4">
         <v>50</v>
       </c>
     </row>
     <row r="46" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C46" s="20"/>
-      <c r="D46" s="21">
+      <c r="C46" s="18"/>
+      <c r="D46" s="19">
         <v>4.3</v>
       </c>
-      <c r="E46" s="21" t="s">
+      <c r="E46" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F46" s="22"/>
-      <c r="G46" s="15">
+      <c r="F46" s="20"/>
+      <c r="G46" s="14">
         <v>2</v>
       </c>
-      <c r="H46" s="16">
+      <c r="H46" s="4">
         <v>4.1</v>
       </c>
-      <c r="I46" s="16"/>
-      <c r="J46" s="16">
+      <c r="I46" s="4"/>
+      <c r="J46" s="4">
         <v>50</v>
       </c>
-      <c r="K46" s="16">
+      <c r="K46" s="4">
         <v>50</v>
       </c>
     </row>
     <row r="47" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C47" s="17"/>
-      <c r="D47" s="18">
+      <c r="C47" s="15"/>
+      <c r="D47" s="16">
         <v>4.4</v>
       </c>
-      <c r="E47" s="18" t="s">
+      <c r="E47" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="F47" s="19"/>
-      <c r="G47" s="15">
+      <c r="F47" s="17"/>
+      <c r="G47" s="14">
         <v>3</v>
       </c>
-      <c r="H47" s="16">
+      <c r="H47" s="4">
         <v>4.2</v>
       </c>
-      <c r="I47" s="16"/>
-      <c r="J47" s="16">
+      <c r="I47" s="4"/>
+      <c r="J47" s="4">
         <v>50</v>
       </c>
-      <c r="K47" s="16">
+      <c r="K47" s="4">
         <v>50</v>
       </c>
     </row>
     <row r="48" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C48" s="20"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="25"/>
-      <c r="H48" s="26"/>
-      <c r="I48" s="26"/>
-      <c r="J48" s="26"/>
-      <c r="K48" s="26"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="21"/>
+      <c r="H48" s="22"/>
+      <c r="I48" s="22"/>
+      <c r="J48" s="22"/>
+      <c r="K48" s="22"/>
     </row>
     <row r="49" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C49" s="17">
+      <c r="C49" s="15">
         <v>5</v>
       </c>
-      <c r="D49" s="18" t="s">
+      <c r="D49" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="E49" s="18"/>
-      <c r="F49" s="19"/>
-      <c r="G49" s="15"/>
-      <c r="H49" s="16"/>
-      <c r="I49" s="16"/>
-      <c r="J49" s="16"/>
-      <c r="K49" s="16"/>
+      <c r="E49" s="16"/>
+      <c r="F49" s="17"/>
+      <c r="G49" s="14"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="4"/>
     </row>
     <row r="50" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C50" s="20"/>
-      <c r="D50" s="21">
+      <c r="C50" s="18"/>
+      <c r="D50" s="19">
         <v>5.1</v>
       </c>
-      <c r="E50" s="21" t="s">
+      <c r="E50" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="F50" s="22"/>
-      <c r="G50" s="15">
+      <c r="F50" s="20"/>
+      <c r="G50" s="14">
         <v>2</v>
       </c>
-      <c r="H50" s="16">
+      <c r="H50" s="4">
         <v>4.4</v>
       </c>
-      <c r="I50" s="16">
+      <c r="I50" s="4">
         <v>50</v>
       </c>
-      <c r="J50" s="16">
+      <c r="J50" s="4">
         <v>50</v>
       </c>
-      <c r="K50" s="16"/>
+      <c r="K50" s="4"/>
     </row>
     <row r="51" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C51" s="17"/>
-      <c r="D51" s="18">
+      <c r="C51" s="15"/>
+      <c r="D51" s="16">
         <v>5.2</v>
       </c>
-      <c r="E51" s="18" t="s">
+      <c r="E51" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="F51" s="19"/>
-      <c r="G51" s="15">
+      <c r="F51" s="17"/>
+      <c r="G51" s="14">
         <v>2</v>
       </c>
-      <c r="H51" s="16">
+      <c r="H51" s="4">
         <v>4.4</v>
       </c>
-      <c r="I51" s="16"/>
-      <c r="J51" s="16"/>
-      <c r="K51" s="16">
+      <c r="I51" s="4"/>
+      <c r="J51" s="4"/>
+      <c r="K51" s="4">
         <v>100</v>
       </c>
     </row>
     <row r="52" ht="22.5" customHeight="1" spans="3:11">
-      <c r="C52" s="28"/>
-      <c r="D52" s="29">
+      <c r="C52" s="23"/>
+      <c r="D52" s="24">
         <v>5.3</v>
       </c>
-      <c r="E52" s="29" t="s">
+      <c r="E52" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F52" s="30"/>
-      <c r="G52" s="15">
+      <c r="F52" s="25"/>
+      <c r="G52" s="14">
         <v>3</v>
       </c>
-      <c r="H52" s="16">
+      <c r="H52" s="4">
         <v>5.1</v>
       </c>
-      <c r="I52" s="16">
+      <c r="I52" s="4">
         <v>34</v>
       </c>
-      <c r="J52" s="16">
+      <c r="J52" s="4">
         <v>33</v>
       </c>
-      <c r="K52" s="16">
+      <c r="K52" s="4">
         <v>33</v>
       </c>
     </row>

</xml_diff>